<commit_message>
Added some keys in config file , change in uploadStorageBucket workflow and also done changes in main.xaml file
</commit_message>
<xml_diff>
--- a/Data/Config.xlsx
+++ b/Data/Config.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://uipath-my.sharepoint.com/personal/alexandra_veizu_uipath_com/Documents/Documents/Projects/REFrameworkNET5/StudioTemplates/REFramework/contentFiles/any/any/pt2/VisualBasic/Data/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="8_{5BECE58B-1E75-461F-92B1-7A9E57B3BB52}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="8_{7381A798-D805-4453-A58C-3183D27A3130}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12576" firstSheet="1" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12576" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Settings" sheetId="1" r:id="rId1"/>
@@ -81,7 +81,7 @@
     <t>Test</t>
   </si>
   <si>
-    <t>EmailResource</t>
+    <t>EmailSource1</t>
   </si>
   <si>
     <t>maheshkothawade47@gmail.com</t>

</xml_diff>